<commit_message>
Apply inbox payloads to workbook
</commit_message>
<xml_diff>
--- a/Wedding_Expense_Tracker_Dec2026.xlsx
+++ b/Wedding_Expense_Tracker_Dec2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nirmal" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Amarai" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deeplaxmie Events" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nirmal's Executive" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Nirmal" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Amarai" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Vendors" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Deeplaxmie Events" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Nirmal's Executive" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vendors'!$A$3:$Q$18</definedName>
@@ -2103,6 +2103,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="49">
       <c r="A3" s="12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Migrate hotel workbook for live room fields
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Wedding_Expense_Tracker_Dec2026.xlsx
+++ b/Wedding_Expense_Tracker_Dec2026.xlsx
@@ -822,16 +822,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:AH64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="49" min="1" max="1"/>
-    <col width="15" customWidth="1" style="49" min="2" max="7"/>
-    <col width="34" customWidth="1" style="49" min="8" max="8"/>
-    <col width="15" customWidth="1" style="49" min="9" max="12"/>
+    <col width="30" customWidth="1" style="49" min="1" max="1"/>
+    <col width="11" customWidth="1" style="49" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="49">
+    <row r="1">
       <c r="A1" s="52" t="inlineStr">
         <is>
           <t>NIRMAL — ROOM PLAN BY NIGHT</t>
@@ -841,11 +839,10 @@
     <row r="2">
       <c r="A2" s="51" t="inlineStr">
         <is>
-          <t>Check-in 08-Dec-2026  |  Check-out 14-Dec-2026  |  10 rooms peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Check-in 08-Dec-2026  |  Check-out 14-Dec-2026  |  10 of 10 rooms booked</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -880,7 +877,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Total rooms</t>
+          <t>Rooms booked</t>
         </is>
       </c>
       <c r="B7" s="4" t="n">
@@ -890,333 +887,310 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
+          <t>Total rooms</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
           <t>Total room-nights</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B9" s="4" t="n">
         <v>37</v>
       </c>
     </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="48" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="48" t="inlineStr">
         <is>
           <t>ROOMS NEEDED PER NIGHT</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="24" customHeight="1" s="49">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Rooms</t>
         </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>08-Dec</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>08-Dec</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>09-Dec</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B14" s="4" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>10-Dec</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B15" s="4" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>11-Dec</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>12-Dec</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="4" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>12-Dec</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t>13-Dec</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B18" s="4" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="7">
-        <f>SUM(B12:B17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" s="48" t="inlineStr">
+      <c r="B19" s="5">
+        <f>SUM(B13:B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="48" t="inlineStr">
         <is>
           <t>ROOM ALLOCATION GRID</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="24" customHeight="1" s="49">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="B21" s="54" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t>Room no.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>08-Dec-2026</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>09-Dec-2026</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>10-Dec-2026</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>11-Dec-2026</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>12-Dec-2026</t>
         </is>
       </c>
-      <c r="H21" s="5" t="inlineStr">
+      <c r="H22" s="5" t="inlineStr">
         <is>
           <t>13-Dec-2026</t>
         </is>
       </c>
-      <c r="I21" s="8" t="inlineStr">
+      <c r="I22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="53" t="inlineStr">
-        <is>
-          <t>Room 1 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B22" s="54" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="53" t="inlineStr">
         <is>
-          <t>Room 2 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B23" s="54" t="n"/>
+          <t>Room 1 - Guest 1</t>
+        </is>
+      </c>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
       <c r="G23" s="9" t="n"/>
       <c r="H23" s="9" t="n"/>
-      <c r="I23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="53" t="inlineStr">
         <is>
-          <t>Room 3 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="n"/>
+          <t>Room 2 - Guest 1</t>
+        </is>
+      </c>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n"/>
-      <c r="I24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="53" t="inlineStr">
         <is>
-          <t>Room 4 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B25" s="54" t="n"/>
+          <t>Room 3 - Guest 1</t>
+        </is>
+      </c>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
       <c r="F25" s="9" t="n"/>
       <c r="G25" s="9" t="n"/>
       <c r="H25" s="9" t="n"/>
-      <c r="I25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="53" t="inlineStr">
         <is>
-          <t>Room 5 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B26" s="54" t="n"/>
+          <t>Room 4 - Guest 1</t>
+        </is>
+      </c>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="9" t="n"/>
       <c r="G26" s="9" t="n"/>
       <c r="H26" s="9" t="n"/>
-      <c r="I26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="53" t="inlineStr">
         <is>
-          <t>Room 6 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B27" s="54" t="n"/>
+          <t>Room 5 - Guest 1</t>
+        </is>
+      </c>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="n"/>
       <c r="G27" s="9" t="n"/>
       <c r="H27" s="9" t="n"/>
-      <c r="I27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="53" t="inlineStr">
         <is>
-          <t>Room 7 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B28" s="54" t="n"/>
+          <t>Room 6 - Guest 1</t>
+        </is>
+      </c>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="9" t="n"/>
       <c r="G28" s="9" t="n"/>
       <c r="H28" s="9" t="n"/>
-      <c r="I28" s="10" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="53" t="inlineStr">
         <is>
-          <t>Room 8 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B29" s="54" t="n"/>
+          <t>Room 7 - Guest 1</t>
+        </is>
+      </c>
       <c r="C29" s="9" t="n"/>
       <c r="D29" s="9" t="n"/>
       <c r="E29" s="9" t="n"/>
       <c r="F29" s="9" t="n"/>
       <c r="G29" s="9" t="n"/>
       <c r="H29" s="9" t="n"/>
-      <c r="I29" s="10" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="53" t="inlineStr">
         <is>
-          <t>Room 9 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B30" s="54" t="n"/>
+          <t>Room 8 - Guest 1</t>
+        </is>
+      </c>
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="9" t="n"/>
       <c r="F30" s="9" t="n"/>
       <c r="G30" s="9" t="n"/>
       <c r="H30" s="9" t="n"/>
-      <c r="I30" s="10" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="53" t="inlineStr">
         <is>
-          <t>Room 10 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B31" s="54" t="n"/>
+          <t>Room 9 - Guest 1</t>
+        </is>
+      </c>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="9" t="n"/>
       <c r="F31" s="9" t="n"/>
       <c r="G31" s="9" t="n"/>
       <c r="H31" s="9" t="n"/>
-      <c r="I31" s="10" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="48" t="inlineStr">
-        <is>
-          <t>SECOND GUEST PER ROOM  -  only fill this block if two people share the room. FILLED counts occupied ROOMS, not guest names.</t>
-        </is>
-      </c>
+      <c r="A32" s="53" t="inlineStr">
+        <is>
+          <t>Room 10 - Guest 1</t>
+        </is>
+      </c>
+      <c r="C32" s="9" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="9" t="n"/>
+      <c r="F32" s="9" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="9" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="53" t="inlineStr">
-        <is>
-          <t>Room 1 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B33" s="54" t="n"/>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
-      <c r="E33" s="9" t="n"/>
-      <c r="F33" s="9" t="n"/>
-      <c r="G33" s="9" t="n"/>
-      <c r="H33" s="9" t="n"/>
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>SECOND GUEST PER ROOM  -  fill only if two people share the room. FILLED counts occupied ROOMS, not guest names.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="53" t="inlineStr">
         <is>
-          <t>Room 2 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B34" s="54" t="n"/>
+          <t>Room 1 - Guest 2</t>
+        </is>
+      </c>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
@@ -1227,10 +1201,9 @@
     <row r="35">
       <c r="A35" s="53" t="inlineStr">
         <is>
-          <t>Room 3 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B35" s="54" t="n"/>
+          <t>Room 2 - Guest 2</t>
+        </is>
+      </c>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="9" t="n"/>
@@ -1238,13 +1211,12 @@
       <c r="G35" s="9" t="n"/>
       <c r="H35" s="9" t="n"/>
     </row>
-    <row r="36" ht="24" customHeight="1" s="49">
+    <row r="36">
       <c r="A36" s="53" t="inlineStr">
         <is>
-          <t>Room 4 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B36" s="54" t="n"/>
+          <t>Room 3 - Guest 2</t>
+        </is>
+      </c>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9" t="n"/>
@@ -1252,13 +1224,12 @@
       <c r="G36" s="9" t="n"/>
       <c r="H36" s="9" t="n"/>
     </row>
-    <row r="37" ht="24" customHeight="1" s="49">
+    <row r="37">
       <c r="A37" s="53" t="inlineStr">
         <is>
-          <t>Room 5 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B37" s="54" t="n"/>
+          <t>Room 4 - Guest 2</t>
+        </is>
+      </c>
       <c r="C37" s="9" t="n"/>
       <c r="D37" s="9" t="n"/>
       <c r="E37" s="9" t="n"/>
@@ -1266,13 +1237,12 @@
       <c r="G37" s="9" t="n"/>
       <c r="H37" s="9" t="n"/>
     </row>
-    <row r="38" ht="24" customHeight="1" s="49">
+    <row r="38">
       <c r="A38" s="53" t="inlineStr">
         <is>
-          <t>Room 6 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B38" s="54" t="n"/>
+          <t>Room 5 - Guest 2</t>
+        </is>
+      </c>
       <c r="C38" s="9" t="n"/>
       <c r="D38" s="9" t="n"/>
       <c r="E38" s="9" t="n"/>
@@ -1280,13 +1250,12 @@
       <c r="G38" s="9" t="n"/>
       <c r="H38" s="9" t="n"/>
     </row>
-    <row r="39" ht="24" customHeight="1" s="49">
+    <row r="39">
       <c r="A39" s="53" t="inlineStr">
         <is>
-          <t>Room 7 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B39" s="54" t="n"/>
+          <t>Room 6 - Guest 2</t>
+        </is>
+      </c>
       <c r="C39" s="9" t="n"/>
       <c r="D39" s="9" t="n"/>
       <c r="E39" s="9" t="n"/>
@@ -1297,10 +1266,9 @@
     <row r="40">
       <c r="A40" s="53" t="inlineStr">
         <is>
-          <t>Room 8 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B40" s="54" t="n"/>
+          <t>Room 7 - Guest 2</t>
+        </is>
+      </c>
       <c r="C40" s="9" t="n"/>
       <c r="D40" s="9" t="n"/>
       <c r="E40" s="9" t="n"/>
@@ -1311,10 +1279,9 @@
     <row r="41">
       <c r="A41" s="53" t="inlineStr">
         <is>
-          <t>Room 9 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B41" s="54" t="n"/>
+          <t>Room 8 - Guest 2</t>
+        </is>
+      </c>
       <c r="C41" s="9" t="n"/>
       <c r="D41" s="9" t="n"/>
       <c r="E41" s="9" t="n"/>
@@ -1325,10 +1292,9 @@
     <row r="42">
       <c r="A42" s="53" t="inlineStr">
         <is>
-          <t>Room 10 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B42" s="54" t="n"/>
+          <t>Room 9 - Guest 2</t>
+        </is>
+      </c>
       <c r="C42" s="9" t="n"/>
       <c r="D42" s="9" t="n"/>
       <c r="E42" s="9" t="n"/>
@@ -1337,170 +1303,344 @@
       <c r="H42" s="9" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="55" t="inlineStr">
+      <c r="A43" s="53" t="inlineStr">
+        <is>
+          <t>Room 10 - Guest 2</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="9" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="48" t="inlineStr">
+        <is>
+          <t>THIRD GUEST PER ROOM  -  fill only if a THIRD person shares the room. These are the extra guests the hotel bills on top of the room rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="53" t="inlineStr">
+        <is>
+          <t>Room 1 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="9" t="n"/>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="9" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="53" t="inlineStr">
+        <is>
+          <t>Room 2 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C46" s="9" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="9" t="n"/>
+      <c r="F46" s="9" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="9" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="53" t="inlineStr">
+        <is>
+          <t>Room 3 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C47" s="9" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="9" t="n"/>
+      <c r="F47" s="9" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="9" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="53" t="inlineStr">
+        <is>
+          <t>Room 4 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="9" t="n"/>
+      <c r="F48" s="9" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="9" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="53" t="inlineStr">
+        <is>
+          <t>Room 5 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="n"/>
+      <c r="D49" s="9" t="n"/>
+      <c r="E49" s="9" t="n"/>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="53" t="inlineStr">
+        <is>
+          <t>Room 6 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="9" t="n"/>
+      <c r="F50" s="9" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="9" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="53" t="inlineStr">
+        <is>
+          <t>Room 7 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="9" t="n"/>
+      <c r="F51" s="9" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="9" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="53" t="inlineStr">
+        <is>
+          <t>Room 8 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="9" t="n"/>
+      <c r="F52" s="9" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="9" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="53" t="inlineStr">
+        <is>
+          <t>Room 9 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="n"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="9" t="n"/>
+      <c r="F53" s="9" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="9" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="53" t="inlineStr">
+        <is>
+          <t>Room 10 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="n"/>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="9" t="n"/>
+      <c r="F54" s="9" t="n"/>
+      <c r="G54" s="9" t="n"/>
+      <c r="H54" s="9" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="55" t="inlineStr">
         <is>
           <t>FILLED</t>
         </is>
       </c>
-      <c r="B43" s="54" t="n"/>
-      <c r="C43" s="11">
-        <f>SUMPRODUCT(--(((C22:C31&lt;&gt;"")+(C33:C42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="D43" s="11">
-        <f>SUMPRODUCT(--(((D22:D31&lt;&gt;"")+(D33:D42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="E43" s="11">
-        <f>SUMPRODUCT(--(((E22:E31&lt;&gt;"")+(E33:E42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="F43" s="11">
-        <f>SUMPRODUCT(--(((F22:F31&lt;&gt;"")+(F33:F42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="G43" s="11">
-        <f>SUMPRODUCT(--(((G22:G31&lt;&gt;"")+(G33:G42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="H43" s="11">
-        <f>SUMPRODUCT(--(((H22:H31&lt;&gt;"")+(H33:H42&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="55" t="inlineStr">
+      <c r="C55" s="11">
+        <f>SUMPRODUCT(--(((C23:C32&lt;&gt;"")+(C34:C43&lt;&gt;"")+(C45:C54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="D55" s="11">
+        <f>SUMPRODUCT(--(((D23:D32&lt;&gt;"")+(D34:D43&lt;&gt;"")+(D45:D54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="E55" s="11">
+        <f>SUMPRODUCT(--(((E23:E32&lt;&gt;"")+(E34:E43&lt;&gt;"")+(E45:E54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="F55" s="11">
+        <f>SUMPRODUCT(--(((F23:F32&lt;&gt;"")+(F34:F43&lt;&gt;"")+(F45:F54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="G55" s="11">
+        <f>SUMPRODUCT(--(((G23:G32&lt;&gt;"")+(G34:G43&lt;&gt;"")+(G45:G54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="H55" s="11">
+        <f>SUMPRODUCT(--(((H23:H32&lt;&gt;"")+(H34:H43&lt;&gt;"")+(H45:H54&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="55" t="inlineStr">
         <is>
           <t>NEEDED</t>
         </is>
       </c>
-      <c r="B44" s="54" t="n"/>
-      <c r="C44" s="11" t="n">
+      <c r="C56" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D44" s="11" t="n">
+      <c r="D56" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="E44" s="11" t="n">
+      <c r="E56" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="F44" s="11" t="n">
+      <c r="F56" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G44" s="11" t="n">
+      <c r="G56" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="H44" s="11" t="n">
+      <c r="H56" s="11" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="55" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="55" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="B45" s="54" t="n"/>
-      <c r="C45" s="4">
-        <f>IF(C43=C44,"OK",IF(C43&lt;C44,"need "&amp;(C44-C43)&amp;" more","extra "&amp;(C43-C44)))</f>
-        <v/>
-      </c>
-      <c r="D45" s="4">
-        <f>IF(D43=D44,"OK",IF(D43&lt;D44,"need "&amp;(D44-D43)&amp;" more","extra "&amp;(D43-D44)))</f>
-        <v/>
-      </c>
-      <c r="E45" s="4">
-        <f>IF(E43=E44,"OK",IF(E43&lt;E44,"need "&amp;(E44-E43)&amp;" more","extra "&amp;(E43-E44)))</f>
-        <v/>
-      </c>
-      <c r="F45" s="4">
-        <f>IF(F43=F44,"OK",IF(F43&lt;F44,"need "&amp;(F44-F43)&amp;" more","extra "&amp;(F43-F44)))</f>
-        <v/>
-      </c>
-      <c r="G45" s="4">
-        <f>IF(G43=G44,"OK",IF(G43&lt;G44,"need "&amp;(G44-G43)&amp;" more","extra "&amp;(G43-G44)))</f>
-        <v/>
-      </c>
-      <c r="H45" s="4">
-        <f>IF(H43=H44,"OK",IF(H43&lt;H44,"need "&amp;(H44-H43)&amp;" more","extra "&amp;(H43-H44)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46"/>
-    <row r="47">
-      <c r="A47" s="50" t="inlineStr">
+      <c r="C57">
+        <f>IF(C55=C56,"OK",IF(C55&lt;C56,"need "&amp;(C56-C55)&amp;" more","extra "&amp;(C55-C56)))</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>IF(D55=D56,"OK",IF(D55&lt;D56,"need "&amp;(D56-D55)&amp;" more","extra "&amp;(D55-D56)))</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>IF(E55=E56,"OK",IF(E55&lt;E56,"need "&amp;(E56-E55)&amp;" more","extra "&amp;(E55-E56)))</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>IF(F55=F56,"OK",IF(F55&lt;F56,"need "&amp;(F56-F55)&amp;" more","extra "&amp;(F55-F56)))</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>IF(G55=G56,"OK",IF(G55&lt;G56,"need "&amp;(G56-G55)&amp;" more","extra "&amp;(G55-G56)))</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>IF(H55=H56,"OK",IF(H55&lt;H56,"need "&amp;(H56-H55)&amp;" more","extra "&amp;(H55-H56)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="55" t="inlineStr">
+        <is>
+          <t>GUESTS</t>
+        </is>
+      </c>
+      <c r="C58" s="11">
+        <f>SUMPRODUCT(--(C23:C32&lt;&gt;""))+SUMPRODUCT(--(C34:C43&lt;&gt;""))+SUMPRODUCT(--(C45:C54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="D58" s="11">
+        <f>SUMPRODUCT(--(D23:D32&lt;&gt;""))+SUMPRODUCT(--(D34:D43&lt;&gt;""))+SUMPRODUCT(--(D45:D54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="E58" s="11">
+        <f>SUMPRODUCT(--(E23:E32&lt;&gt;""))+SUMPRODUCT(--(E34:E43&lt;&gt;""))+SUMPRODUCT(--(E45:E54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="F58" s="11">
+        <f>SUMPRODUCT(--(F23:F32&lt;&gt;""))+SUMPRODUCT(--(F34:F43&lt;&gt;""))+SUMPRODUCT(--(F45:F54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="G58" s="11">
+        <f>SUMPRODUCT(--(G23:G32&lt;&gt;""))+SUMPRODUCT(--(G34:G43&lt;&gt;""))+SUMPRODUCT(--(G45:G54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="H58" s="11">
+        <f>SUMPRODUCT(--(H23:H32&lt;&gt;""))+SUMPRODUCT(--(H34:H43&lt;&gt;""))+SUMPRODUCT(--(H45:H54&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="55" t="inlineStr">
+        <is>
+          <t>3rd GUESTS</t>
+        </is>
+      </c>
+      <c r="C59" s="11">
+        <f>SUMPRODUCT(--(C45:C54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="D59" s="11">
+        <f>SUMPRODUCT(--(D45:D54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="E59" s="11">
+        <f>SUMPRODUCT(--(E45:E54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="F59" s="11">
+        <f>SUMPRODUCT(--(F45:F54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="G59" s="11">
+        <f>SUMPRODUCT(--(G45:G54&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="H59" s="11">
+        <f>SUMPRODUCT(--(H45:H54&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="50" t="inlineStr">
         <is>
           <t>How to use:  every room has a 'Guest 1' row and a 'Guest 2' row. Type a name in the white cell for the night that guest is staying. Leave a cell blank if that guest is not in that room that night. FILLED counts occupied ROOMS, not guest names, so a room with two guests still counts as one room.</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="50" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="50" t="inlineStr">
         <is>
           <t>Give this grid to the front desk on arrival. Hand out room keys against the names you typed.</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="50" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="50" t="inlineStr">
         <is>
           <t>Two guests in one room?  Put the first name in the 'Guest 1' row and the second in the 'Guest 2' row for that same night. Both rows belong to the same room, so it still counts as one room against NEEDED.</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="50" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="50" t="inlineStr">
         <is>
           <t>Check-out is 14-Dec-2026. 13-Dec is the last night and only 2 rooms are needed, so release the other 8 rooms after checkout on 13-Dec.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="32">
-    <mergeCell ref="A48:H48"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A49:H49"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A50:H50"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A43:B43"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A34:B34"/>
+  <mergeCells count="9">
+    <mergeCell ref="A21:AH21"/>
+    <mergeCell ref="A63:AH63"/>
+    <mergeCell ref="A64:AH64"/>
+    <mergeCell ref="A33:AH33"/>
+    <mergeCell ref="A11:AH11"/>
+    <mergeCell ref="A44:AH44"/>
+    <mergeCell ref="A61:AH61"/>
+    <mergeCell ref="A4:AH4"/>
+    <mergeCell ref="A62:AH62"/>
   </mergeCells>
-  <conditionalFormatting sqref="C45:H45">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>ISNUMBER(SEARCH("need",C34))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
-      <formula>ISNUMBER(SEARCH("over",C34))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1511,16 +1651,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:AG56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" style="49" min="1" max="1"/>
-    <col width="15" customWidth="1" style="49" min="2" max="5"/>
-    <col width="34" customWidth="1" style="49" min="6" max="6"/>
-    <col width="15" customWidth="1" style="49" min="7" max="12"/>
+    <col width="30" customWidth="1" style="49" min="1" max="1"/>
+    <col width="11" customWidth="1" style="49" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="21" customHeight="1" s="49">
+    <row r="1">
       <c r="A1" s="52" t="inlineStr">
         <is>
           <t>AMARAI — ROOM PLAN BY NIGHT</t>
@@ -1530,11 +1668,10 @@
     <row r="2">
       <c r="A2" s="51" t="inlineStr">
         <is>
-          <t>Check-in 08-Dec-2026  |  Check-out 12-Dec-2026 at 12:30 PM  |  7 rooms peak</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
+          <t>Check-in 08-Dec-2026  |  Check-out 12-Dec-2026  |  7 of 7 rooms booked</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -1581,7 +1718,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Total rooms</t>
+          <t>Rooms booked</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
@@ -1591,330 +1728,309 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
+          <t>Total rooms</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Total room-nights</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B10" s="4" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
-      <c r="A11" s="48" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="48" t="inlineStr">
         <is>
           <t>ROOMS NEEDED PER NIGHT</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="24" customHeight="1" s="49">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>Rooms</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>08-Dec</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B14" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>09-Dec</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B15" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>10-Dec</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B16" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>11-Dec</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B17" t="n">
         <v>7</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>12-Dec</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B18" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="7">
-        <f>SUM(B13:B17)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19"/>
-    <row r="20" ht="24" customHeight="1" s="49">
-      <c r="A20" s="48" t="inlineStr">
+      <c r="B19" s="5">
+        <f>SUM(B14:B18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="48" t="inlineStr">
         <is>
           <t>ROOM ALLOCATION GRID</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="56" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="56" t="inlineStr">
         <is>
           <t>Room</t>
         </is>
       </c>
-      <c r="B21" s="54" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B22" s="56" t="inlineStr">
+        <is>
+          <t>Room no.</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>08-Dec-2026</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>09-Dec-2026</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E22" s="5" t="inlineStr">
         <is>
           <t>10-Dec-2026</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F22" s="5" t="inlineStr">
         <is>
           <t>11-Dec-2026</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>12-Dec-2026</t>
         </is>
       </c>
-      <c r="H21" s="8" t="inlineStr">
+      <c r="H22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="53" t="inlineStr">
-        <is>
-          <t>Room 1 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B22" s="54" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="10" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="53" t="inlineStr">
         <is>
-          <t>Room 2 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B23" s="54" t="n"/>
+          <t>Room 1 - Guest 1</t>
+        </is>
+      </c>
       <c r="C23" s="9" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="9" t="n"/>
       <c r="F23" s="9" t="n"/>
       <c r="G23" s="9" t="n"/>
-      <c r="H23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="53" t="inlineStr">
         <is>
-          <t>Room 3 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B24" s="54" t="n"/>
+          <t>Room 2 - Guest 1</t>
+        </is>
+      </c>
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
       <c r="F24" s="9" t="n"/>
       <c r="G24" s="9" t="n"/>
-      <c r="H24" s="10" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="53" t="inlineStr">
         <is>
-          <t>Room 4 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B25" s="54" t="n"/>
+          <t>Room 3 - Guest 1</t>
+        </is>
+      </c>
       <c r="C25" s="9" t="n"/>
       <c r="D25" s="9" t="n"/>
       <c r="E25" s="9" t="n"/>
       <c r="F25" s="9" t="n"/>
       <c r="G25" s="9" t="n"/>
-      <c r="H25" s="10" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="53" t="inlineStr">
         <is>
-          <t>Room 5 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B26" s="54" t="n"/>
+          <t>Room 4 - Guest 1</t>
+        </is>
+      </c>
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
       <c r="F26" s="9" t="n"/>
       <c r="G26" s="9" t="n"/>
-      <c r="H26" s="10" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="53" t="inlineStr">
         <is>
-          <t>Room 6 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B27" s="54" t="n"/>
+          <t>Room 5 - Guest 1</t>
+        </is>
+      </c>
       <c r="C27" s="9" t="n"/>
       <c r="D27" s="9" t="n"/>
       <c r="E27" s="9" t="n"/>
       <c r="F27" s="9" t="n"/>
       <c r="G27" s="9" t="n"/>
-      <c r="H27" s="10" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="53" t="inlineStr">
         <is>
-          <t>Room 7 - Guest 1</t>
-        </is>
-      </c>
-      <c r="B28" s="54" t="n"/>
+          <t>Room 6 - Guest 1</t>
+        </is>
+      </c>
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
       <c r="F28" s="9" t="n"/>
       <c r="G28" s="9" t="n"/>
-      <c r="H28" s="10" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="48" t="inlineStr">
-        <is>
-          <t>SECOND GUEST PER ROOM  -  only fill this block if two people share the room. FILLED counts occupied ROOMS, not guest names.</t>
-        </is>
-      </c>
+      <c r="A29" s="53" t="inlineStr">
+        <is>
+          <t>Room 7 - Guest 1</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="53" t="inlineStr">
-        <is>
-          <t>Room 1 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B30" s="54" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
-      <c r="G30" s="9" t="n"/>
+      <c r="A30" s="48" t="inlineStr">
+        <is>
+          <t>SECOND GUEST PER ROOM  -  fill only if two people share the room. FILLED counts occupied ROOMS, not guest names.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="53" t="inlineStr">
         <is>
-          <t>Room 2 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B31" s="54" t="n"/>
+          <t>Room 1 - Guest 2</t>
+        </is>
+      </c>
       <c r="C31" s="9" t="n"/>
       <c r="D31" s="9" t="n"/>
       <c r="E31" s="9" t="n"/>
       <c r="F31" s="9" t="n"/>
       <c r="G31" s="9" t="n"/>
     </row>
-    <row r="32" ht="24" customHeight="1" s="49">
+    <row r="32">
       <c r="A32" s="53" t="inlineStr">
         <is>
-          <t>Room 3 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B32" s="54" t="n"/>
+          <t>Room 2 - Guest 2</t>
+        </is>
+      </c>
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
       <c r="F32" s="9" t="n"/>
       <c r="G32" s="9" t="n"/>
     </row>
-    <row r="33" ht="24" customHeight="1" s="49">
+    <row r="33">
       <c r="A33" s="53" t="inlineStr">
         <is>
-          <t>Room 4 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B33" s="54" t="n"/>
+          <t>Room 3 - Guest 2</t>
+        </is>
+      </c>
       <c r="C33" s="9" t="n"/>
       <c r="D33" s="9" t="n"/>
       <c r="E33" s="9" t="n"/>
       <c r="F33" s="9" t="n"/>
       <c r="G33" s="9" t="n"/>
     </row>
-    <row r="34" ht="24" customHeight="1" s="49">
+    <row r="34">
       <c r="A34" s="53" t="inlineStr">
         <is>
-          <t>Room 5 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B34" s="54" t="n"/>
+          <t>Room 4 - Guest 2</t>
+        </is>
+      </c>
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
       <c r="F34" s="9" t="n"/>
       <c r="G34" s="9" t="n"/>
     </row>
-    <row r="35" ht="24" customHeight="1" s="49">
+    <row r="35">
       <c r="A35" s="53" t="inlineStr">
         <is>
-          <t>Room 6 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B35" s="54" t="n"/>
+          <t>Room 5 - Guest 2</t>
+        </is>
+      </c>
       <c r="C35" s="9" t="n"/>
       <c r="D35" s="9" t="n"/>
       <c r="E35" s="9" t="n"/>
       <c r="F35" s="9" t="n"/>
       <c r="G35" s="9" t="n"/>
     </row>
-    <row r="36" ht="24" customHeight="1" s="49">
+    <row r="36">
       <c r="A36" s="53" t="inlineStr">
         <is>
-          <t>Room 7 - Guest 2</t>
-        </is>
-      </c>
-      <c r="B36" s="54" t="n"/>
+          <t>Room 6 - Guest 2</t>
+        </is>
+      </c>
       <c r="C36" s="9" t="n"/>
       <c r="D36" s="9" t="n"/>
       <c r="E36" s="9" t="n"/>
@@ -1922,161 +2038,286 @@
       <c r="G36" s="9" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="55" t="inlineStr">
+      <c r="A37" s="53" t="inlineStr">
+        <is>
+          <t>Room 7 - Guest 2</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>THIRD GUEST PER ROOM  -  fill only if a THIRD person shares the room. These are the extra guests the hotel bills on top of the room rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="53" t="inlineStr">
+        <is>
+          <t>Room 1 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C39" s="9" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="9" t="n"/>
+      <c r="F39" s="9" t="n"/>
+      <c r="G39" s="9" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="53" t="inlineStr">
+        <is>
+          <t>Room 2 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="9" t="n"/>
+      <c r="F40" s="9" t="n"/>
+      <c r="G40" s="9" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="53" t="inlineStr">
+        <is>
+          <t>Room 3 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C41" s="9" t="n"/>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="9" t="n"/>
+      <c r="F41" s="9" t="n"/>
+      <c r="G41" s="9" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="53" t="inlineStr">
+        <is>
+          <t>Room 4 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="9" t="n"/>
+      <c r="F42" s="9" t="n"/>
+      <c r="G42" s="9" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="53" t="inlineStr">
+        <is>
+          <t>Room 5 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C43" s="9" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="9" t="n"/>
+      <c r="F43" s="9" t="n"/>
+      <c r="G43" s="9" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="53" t="inlineStr">
+        <is>
+          <t>Room 6 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C44" s="9" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="9" t="n"/>
+      <c r="G44" s="9" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="53" t="inlineStr">
+        <is>
+          <t>Room 7 - Guest 3</t>
+        </is>
+      </c>
+      <c r="C45" s="9" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="9" t="n"/>
+      <c r="F45" s="9" t="n"/>
+      <c r="G45" s="9" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="55" t="inlineStr">
         <is>
           <t>FILLED</t>
         </is>
       </c>
-      <c r="B37" s="54" t="n"/>
-      <c r="C37" s="9">
-        <f>SUMPRODUCT(--(((C22:C28&lt;&gt;"")+(C30:C36&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="D37" s="11">
-        <f>SUMPRODUCT(--(((D22:D28&lt;&gt;"")+(D30:D36&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="E37" s="11">
-        <f>SUMPRODUCT(--(((E22:E28&lt;&gt;"")+(E30:E36&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="F37" s="11">
-        <f>SUMPRODUCT(--(((F22:F28&lt;&gt;"")+(F30:F36&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-      <c r="G37" s="11">
-        <f>SUMPRODUCT(--(((G22:G28&lt;&gt;"")+(G30:G36&lt;&gt;""))&gt;0))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="55" t="inlineStr">
+      <c r="C46" s="9">
+        <f>SUMPRODUCT(--(((C23:C29&lt;&gt;"")+(C31:C37&lt;&gt;"")+(C39:C45&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="D46" s="9">
+        <f>SUMPRODUCT(--(((D23:D29&lt;&gt;"")+(D31:D37&lt;&gt;"")+(D39:D45&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="E46" s="9">
+        <f>SUMPRODUCT(--(((E23:E29&lt;&gt;"")+(E31:E37&lt;&gt;"")+(E39:E45&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="F46" s="9">
+        <f>SUMPRODUCT(--(((F23:F29&lt;&gt;"")+(F31:F37&lt;&gt;"")+(F39:F45&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+      <c r="G46" s="9">
+        <f>SUMPRODUCT(--(((G23:G29&lt;&gt;"")+(G31:G37&lt;&gt;"")+(G39:G45&lt;&gt;""))&gt;0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="55" t="inlineStr">
         <is>
           <t>NEEDED</t>
         </is>
       </c>
-      <c r="B38" s="54" t="n"/>
-      <c r="C38" s="9" t="n">
+      <c r="C47" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="D38" s="11" t="n">
+      <c r="D47" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="E38" s="11" t="n">
+      <c r="E47" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="F38" s="11" t="n">
+      <c r="F47" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="G38" s="11" t="n">
+      <c r="G47" s="9" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="55" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="55" t="inlineStr">
         <is>
           <t>STATUS</t>
         </is>
       </c>
-      <c r="B39" s="54" t="n"/>
-      <c r="C39" s="9">
-        <f>IF(C37=C38,"OK",IF(C37&lt;C38,"need "&amp;(C38-C37)&amp;" more","extra "&amp;(C37-C38)))</f>
-        <v/>
-      </c>
-      <c r="D39" s="4">
-        <f>IF(D37=D38,"OK",IF(D37&lt;D38,"need "&amp;(D38-D37)&amp;" more","extra "&amp;(D37-D38)))</f>
-        <v/>
-      </c>
-      <c r="E39" s="4">
-        <f>IF(E37=E38,"OK",IF(E37&lt;E38,"need "&amp;(E38-E37)&amp;" more","extra "&amp;(E37-E38)))</f>
-        <v/>
-      </c>
-      <c r="F39" s="4">
-        <f>IF(F37=F38,"OK",IF(F37&lt;F38,"need "&amp;(F38-F37)&amp;" more","extra "&amp;(F37-F38)))</f>
-        <v/>
-      </c>
-      <c r="G39" s="4">
-        <f>IF(G37=G38,"OK",IF(G37&lt;G38,"need "&amp;(G38-G37)&amp;" more","extra "&amp;(G37-G38)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40"/>
-    <row r="41">
-      <c r="A41" s="50" t="inlineStr">
+      <c r="C48">
+        <f>IF(C46=C47,"OK",IF(C46&lt;C47,"need "&amp;(C47-C46)&amp;" more","extra "&amp;(C46-C47)))</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>IF(D46=D47,"OK",IF(D46&lt;D47,"need "&amp;(D47-D46)&amp;" more","extra "&amp;(D46-D47)))</f>
+        <v/>
+      </c>
+      <c r="E48">
+        <f>IF(E46=E47,"OK",IF(E46&lt;E47,"need "&amp;(E47-E46)&amp;" more","extra "&amp;(E46-E47)))</f>
+        <v/>
+      </c>
+      <c r="F48">
+        <f>IF(F46=F47,"OK",IF(F46&lt;F47,"need "&amp;(F47-F46)&amp;" more","extra "&amp;(F46-F47)))</f>
+        <v/>
+      </c>
+      <c r="G48">
+        <f>IF(G46=G47,"OK",IF(G46&lt;G47,"need "&amp;(G47-G46)&amp;" more","extra "&amp;(G46-G47)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="55" t="inlineStr">
+        <is>
+          <t>GUESTS</t>
+        </is>
+      </c>
+      <c r="C49" s="9">
+        <f>SUMPRODUCT(--(C23:C29&lt;&gt;""))+SUMPRODUCT(--(C31:C37&lt;&gt;""))+SUMPRODUCT(--(C39:C45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="D49" s="9">
+        <f>SUMPRODUCT(--(D23:D29&lt;&gt;""))+SUMPRODUCT(--(D31:D37&lt;&gt;""))+SUMPRODUCT(--(D39:D45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="E49" s="9">
+        <f>SUMPRODUCT(--(E23:E29&lt;&gt;""))+SUMPRODUCT(--(E31:E37&lt;&gt;""))+SUMPRODUCT(--(E39:E45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="F49" s="9">
+        <f>SUMPRODUCT(--(F23:F29&lt;&gt;""))+SUMPRODUCT(--(F31:F37&lt;&gt;""))+SUMPRODUCT(--(F39:F45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="G49" s="9">
+        <f>SUMPRODUCT(--(G23:G29&lt;&gt;""))+SUMPRODUCT(--(G31:G37&lt;&gt;""))+SUMPRODUCT(--(G39:G45&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="55" t="inlineStr">
+        <is>
+          <t>3rd GUESTS</t>
+        </is>
+      </c>
+      <c r="C50" s="9">
+        <f>SUMPRODUCT(--(C39:C45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="D50" s="9">
+        <f>SUMPRODUCT(--(D39:D45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="E50" s="9">
+        <f>SUMPRODUCT(--(E39:E45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="F50" s="9">
+        <f>SUMPRODUCT(--(F39:F45&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="G50" s="9">
+        <f>SUMPRODUCT(--(G39:G45&lt;&gt;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="50" t="inlineStr">
         <is>
           <t>How to use:  every room has a 'Guest 1' row and a 'Guest 2' row. Type a name in the white cell for the night that guest is staying. Leave a cell blank if that guest is not in that room that night. FILLED counts occupied ROOMS, not guest names, so a room with two guests still counts as one room.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="50" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="50" t="inlineStr">
         <is>
           <t>Give this grid to the front desk on arrival. Hand out room keys against the names you typed.</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="50" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="50" t="inlineStr">
         <is>
           <t>Two guests in one room?  Put the first name in the 'Guest 1' row and the second in the 'Guest 2' row for that same night. Both rows belong to the same room, so it still counts as one room against NEEDED.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="50" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="50" t="inlineStr">
         <is>
           <t>Checkout is 12-Dec at 12:30 PM, so 12-Dec needs 0 rooms overnight. Rooms 1-7 are held for the nights of 08, 09, 10 and 11 Dec only.</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="50" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="50" t="inlineStr">
         <is>
           <t>Ask the front desk to release all 7 rooms on 12-Dec at 12:30 PM. Only 2 of the 7 rooms are actually needed on the night of 08-Dec.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A4:G4"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A44:G44"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A45:G45"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A41:G41"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A34:B34"/>
+  <mergeCells count="10">
+    <mergeCell ref="A56:AG56"/>
+    <mergeCell ref="A21:AG21"/>
+    <mergeCell ref="A53:AG53"/>
+    <mergeCell ref="A55:AG55"/>
+    <mergeCell ref="A12:AG12"/>
+    <mergeCell ref="A4:AG4"/>
+    <mergeCell ref="A38:AG38"/>
+    <mergeCell ref="A30:AG30"/>
+    <mergeCell ref="A54:AG54"/>
+    <mergeCell ref="A52:AG52"/>
   </mergeCells>
-  <conditionalFormatting sqref="C39:G39">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="2">
-      <formula>"OK"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="0">
-      <formula>ISNUMBER(SEARCH("need",D30))</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="1">
-      <formula>ISNUMBER(SEARCH("over",D30))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2111,7 +2352,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="30" customHeight="1" s="49">
       <c r="A3" s="12" t="inlineStr">
         <is>

</xml_diff>